<commit_message>
Actualizar plantilla del inventario: subcategoría, garantía, marcas y tasa de $3.000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cartago_Inventario_Plantilla.xlsx
+++ b/docs/Cartago_Inventario_Plantilla.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Productos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Variantes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Imagenes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Configuracion" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Listas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variantes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imagenes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marcas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,7 +124,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -221,45 +222,65 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Código corto y único: letra de la categoría + número (m1, c1). No se repite ni se cambia.</t>
+        <t>Código corto y único: letra + número (m1, e1, j1). No se repite ni se cambia.</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Elige de la lista (pestaña Listas).</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Elige de la lista. Debe corresponder a la categoría (ver pestaña Listas).</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Elige de la lista (pestaña Marcas). Cada producto muestra el logo de su marca.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Pesos colombianos, sin puntos ni signo. 0 o vacío = Precio a consultar.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Opcional. Precio fijo en dólares. Vacío = se convierte con la tasa de Configuracion.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>SI = se ve en la página. NO = escondido.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>SI = aparece en Productos destacados de la página de inicio.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>SI = el cliente puede escribir iniciales, medidas o repujado.</t>
+        <t>SI = el cliente puede escribir el bordado o el detalle que quiere.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>Texto de ayuda que ve el cliente en el campo de personalización.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Texto resaltado en la ficha del producto.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>Se calcula solo: suma del stock de todos los colores en Variantes.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Se calcula solo: cuántas fotos tiene el producto en Imagenes.</t>
       </text>
@@ -281,7 +302,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Código único de esta variante: id + 3 letras del color (c1-NEG). Sin colores: el mismo id.</t>
+        <t>Código único de esta variante: id + 3 letras del color (j2-NEG). Sin colores: el mismo id.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -316,7 +337,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Nombre del archivo en la carpeta de Drive, para ubicarlo (c1-1.jpg).</t>
+        <t>Nombre del archivo en la carpeta de Drive, para ubicarlo (e2-1.jpg).</t>
       </text>
     </comment>
   </commentList>
@@ -331,7 +352,32 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Categorías que se pueden elegir en Productos. Agreguen o cambien aquí.</t>
+        <t>Nombre de la marca tal como se escribe en Productos.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Link del logo. Cartago, San Fermín y Mesacé ya vienen incluidos en la página.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>JCS Emprende</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Categorías que se pueden elegir en Productos.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Subcategorías que se pueden elegir en Productos.</t>
       </text>
     </comment>
   </commentList>
@@ -627,11 +673,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B29"/>
+  <dimension ref="B2:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
@@ -661,7 +707,7 @@
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Productos: una fila por producto (nombre, categoría, descripción, precio).</t>
+          <t>Productos: una fila por producto (nombre, categoría, subcategoría, marca, descripción, precio).</t>
         </is>
       </c>
     </row>
@@ -682,129 +728,150 @@
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Configuracion: ajustes generales, como la tasa de cambio para los precios en dólares.</t>
+          <t>Marcas: las marcas que vende Cartago y el link de su logo (opcional).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Listas: categorías permitidas. Si agregan una categoría nueva, escríbanla ahí primero.</t>
+          <t>Configuracion: la tasa del dólar. Se actualiza cada 8 días.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Listas: categorías y subcategorías permitidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Cómo llenar</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>1. La fila 2 de cada pestaña (en rosado) es un ejemplo. Escriban debajo de ella y bórrenla cuando carguen el primer producto real.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2. Cada producto tiene un id corto y único: una letra de la categoría y un número (m1, m2 para monturas; c1 para correas). Nunca reutilicen un id.</t>
+          <t>1. La fila 2 de cada pestaña (en rosado) es un ejemplo. Bórrenla cuando carguen el primer producto real: si no, aparece en la página.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>3. Precio en pesos sin puntos ni signo: 85000. Si el precio es 0 o se deja vacío, la página muestra "Precio a consultar".</t>
+          <t>2. Cada producto tiene un id corto y único: una letra y un número (m1, m2 para monturas; e1 para equino; j1 para jinete). Nunca reutilicen un id.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>4. precio_usd es opcional: llénenlo solo si quieren un precio fijo en dólares. Si queda vacío, se calcula con la tasa de Configuracion.</t>
+          <t>3. Categoría y subcategoría se eligen de la lista. Ej.: Equino &gt; Cabeza para aperos, jáquimas, riendas y frenos.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>5. activo = NO esconde el producto de la página sin borrarlo. destacado = SI lo muestra en la página de inicio.</t>
+          <t>4. Precio en pesos sin puntos ni signo: 85000. Precio 0 o vacío = "Precio a consultar" (silla mexicana, frenos a la medida, Chaparral personalizada...).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>6. personalizable = SI muestra un campo para que el cliente escriba iniciales, medidas o repujado. nota_personalizacion es la pista que ve el cliente.</t>
+          <t>5. precio_usd es opcional: solo si quieren un precio fijo en dólares. Si queda vacío, se calcula con la tasa de Configuracion.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>7. En Variantes, si el producto no maneja colores, dejen una sola fila con el color vacío. Con stock 0 el color aparece como agotado.</t>
+          <t>6. activo = NO esconde el producto sin borrarlo. destacado = SI lo muestra en la página de inicio.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>8. Las columnas grises en cursiva (stock_total, fotos) se calculan solas: no las escriban. Vienen listas para 150 productos; si pasan de ahí, copien la última fórmula hacia abajo.</t>
+          <t>7. personalizable = SI muestra un campo para que el cliente escriba el bordado (nombre del caballo, criadero o iniciales). nota_personalizacion es la pista que ve el cliente.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Fotos</t>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>8. garantia es opcional: un texto que aparece resaltado en la ficha. Ej.: la garantía de cambio de los frenos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>9. En Variantes, si el producto no maneja colores, dejen una sola fila con el color vacío. Con stock 0 el color aparece como agotado.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Suban las fotos a la carpeta "Fotos de productos" de este mismo Drive, nombradas con el id del producto y un número: c1-1.jpg, c1-2.jpg.</t>
+          <t>10. Las columnas grises en cursiva (stock_total, fotos) se calculan solas. Vienen listas para 150 productos; si pasan de ahí, copien la última fórmula hacia abajo.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>JCS Emprende las optimiza y escribe el link en la pestaña Imagenes. Fotos de buena luz, fondo limpio y al menos 1200 px de lado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Al vender</t>
+      <c r="B24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Fotos</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Suban las fotos a la carpeta "Fotos de productos" de este mismo Drive, nombradas con el id del producto y un número: e2-1.jpg, e2-2.jpg.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Cuando el cliente pague, resten las unidades vendidas en la columna stock de la pestaña Variantes.</t>
+          <t>JCS Emprende las optimiza y escribe el link en la pestaña Imagenes. Buena luz, fondo limpio y al menos 1200 px de lado.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="3" t="inlineStr"/>
     </row>
-    <row r="29">
-      <c r="B29" s="5" t="inlineStr">
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Al vender</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Cuando el cliente pague, resten las unidades vendidas en la columna stock de la pestaña Variantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>No cambien los nombres de las pestañas ni de los encabezados: la página los usa para leer los datos.</t>
         </is>
@@ -821,22 +888,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M151"/>
+  <dimension ref="A1:O151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -857,50 +926,60 @@
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
+          <t>subcategoria</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
           <t>marca</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>precio_usd</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>destacado</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>personalizable</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>nota_personalizacion</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>garantia</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>stock_total</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>fotos</t>
         </is>
@@ -909,1564 +988,1574 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>e2</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Correa clásica</t>
+          <t>Freno a la medida</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Correas</t>
+          <t>Equino</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
+          <t>Cabeza</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
           <t>Cartago</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>Correa en cuero de una sola pieza, 3,5 cm de ancho, hebilla en acero envejecido.</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="n">
-        <v>85000</v>
-      </c>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Freno fabricado bajo medida para tu caballo.</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K2" s="8" t="inlineStr">
-        <is>
-          <t>Indícanos la talla de cintura y si quieres iniciales grabadas.</t>
-        </is>
-      </c>
-      <c r="L2" s="10">
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>Garantía de cambio: lo ensayas y, si no se le acomoda a tu caballo, te lo cambiamos sin costo adicional.</t>
+        </is>
+      </c>
+      <c r="N2" s="10">
         <f>IF(A2="","",SUMIF(Variantes!A:A,A2,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M2" s="10">
+      <c r="O2" s="10">
         <f>IF(A2="","",COUNTIF(Imagenes!A:A,A2))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="L3" s="10">
+      <c r="N3" s="10">
         <f>IF(A3="","",SUMIF(Variantes!A:A,A3,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M3" s="10">
+      <c r="O3" s="10">
         <f>IF(A3="","",COUNTIF(Imagenes!A:A,A3))</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="L4" s="10">
+      <c r="N4" s="10">
         <f>IF(A4="","",SUMIF(Variantes!A:A,A4,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M4" s="10">
+      <c r="O4" s="10">
         <f>IF(A4="","",COUNTIF(Imagenes!A:A,A4))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="L5" s="10">
+      <c r="N5" s="10">
         <f>IF(A5="","",SUMIF(Variantes!A:A,A5,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M5" s="10">
+      <c r="O5" s="10">
         <f>IF(A5="","",COUNTIF(Imagenes!A:A,A5))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="L6" s="10">
+      <c r="N6" s="10">
         <f>IF(A6="","",SUMIF(Variantes!A:A,A6,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M6" s="10">
+      <c r="O6" s="10">
         <f>IF(A6="","",COUNTIF(Imagenes!A:A,A6))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="L7" s="10">
+      <c r="N7" s="10">
         <f>IF(A7="","",SUMIF(Variantes!A:A,A7,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M7" s="10">
+      <c r="O7" s="10">
         <f>IF(A7="","",COUNTIF(Imagenes!A:A,A7))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="L8" s="10">
+      <c r="N8" s="10">
         <f>IF(A8="","",SUMIF(Variantes!A:A,A8,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M8" s="10">
+      <c r="O8" s="10">
         <f>IF(A8="","",COUNTIF(Imagenes!A:A,A8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="L9" s="10">
+      <c r="N9" s="10">
         <f>IF(A9="","",SUMIF(Variantes!A:A,A9,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M9" s="10">
+      <c r="O9" s="10">
         <f>IF(A9="","",COUNTIF(Imagenes!A:A,A9))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="L10" s="10">
+      <c r="N10" s="10">
         <f>IF(A10="","",SUMIF(Variantes!A:A,A10,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M10" s="10">
+      <c r="O10" s="10">
         <f>IF(A10="","",COUNTIF(Imagenes!A:A,A10))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="L11" s="10">
+      <c r="N11" s="10">
         <f>IF(A11="","",SUMIF(Variantes!A:A,A11,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M11" s="10">
+      <c r="O11" s="10">
         <f>IF(A11="","",COUNTIF(Imagenes!A:A,A11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="L12" s="10">
+      <c r="N12" s="10">
         <f>IF(A12="","",SUMIF(Variantes!A:A,A12,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M12" s="10">
+      <c r="O12" s="10">
         <f>IF(A12="","",COUNTIF(Imagenes!A:A,A12))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="L13" s="10">
+      <c r="N13" s="10">
         <f>IF(A13="","",SUMIF(Variantes!A:A,A13,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M13" s="10">
+      <c r="O13" s="10">
         <f>IF(A13="","",COUNTIF(Imagenes!A:A,A13))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="L14" s="10">
+      <c r="N14" s="10">
         <f>IF(A14="","",SUMIF(Variantes!A:A,A14,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M14" s="10">
+      <c r="O14" s="10">
         <f>IF(A14="","",COUNTIF(Imagenes!A:A,A14))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="L15" s="10">
+      <c r="N15" s="10">
         <f>IF(A15="","",SUMIF(Variantes!A:A,A15,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M15" s="10">
+      <c r="O15" s="10">
         <f>IF(A15="","",COUNTIF(Imagenes!A:A,A15))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="L16" s="10">
+      <c r="N16" s="10">
         <f>IF(A16="","",SUMIF(Variantes!A:A,A16,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M16" s="10">
+      <c r="O16" s="10">
         <f>IF(A16="","",COUNTIF(Imagenes!A:A,A16))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="L17" s="10">
+      <c r="N17" s="10">
         <f>IF(A17="","",SUMIF(Variantes!A:A,A17,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M17" s="10">
+      <c r="O17" s="10">
         <f>IF(A17="","",COUNTIF(Imagenes!A:A,A17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="L18" s="10">
+      <c r="N18" s="10">
         <f>IF(A18="","",SUMIF(Variantes!A:A,A18,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M18" s="10">
+      <c r="O18" s="10">
         <f>IF(A18="","",COUNTIF(Imagenes!A:A,A18))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="L19" s="10">
+      <c r="N19" s="10">
         <f>IF(A19="","",SUMIF(Variantes!A:A,A19,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M19" s="10">
+      <c r="O19" s="10">
         <f>IF(A19="","",COUNTIF(Imagenes!A:A,A19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="L20" s="10">
+      <c r="N20" s="10">
         <f>IF(A20="","",SUMIF(Variantes!A:A,A20,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M20" s="10">
+      <c r="O20" s="10">
         <f>IF(A20="","",COUNTIF(Imagenes!A:A,A20))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="L21" s="10">
+      <c r="N21" s="10">
         <f>IF(A21="","",SUMIF(Variantes!A:A,A21,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M21" s="10">
+      <c r="O21" s="10">
         <f>IF(A21="","",COUNTIF(Imagenes!A:A,A21))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="L22" s="10">
+      <c r="N22" s="10">
         <f>IF(A22="","",SUMIF(Variantes!A:A,A22,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M22" s="10">
+      <c r="O22" s="10">
         <f>IF(A22="","",COUNTIF(Imagenes!A:A,A22))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="L23" s="10">
+      <c r="N23" s="10">
         <f>IF(A23="","",SUMIF(Variantes!A:A,A23,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M23" s="10">
+      <c r="O23" s="10">
         <f>IF(A23="","",COUNTIF(Imagenes!A:A,A23))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="L24" s="10">
+      <c r="N24" s="10">
         <f>IF(A24="","",SUMIF(Variantes!A:A,A24,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M24" s="10">
+      <c r="O24" s="10">
         <f>IF(A24="","",COUNTIF(Imagenes!A:A,A24))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="L25" s="10">
+      <c r="N25" s="10">
         <f>IF(A25="","",SUMIF(Variantes!A:A,A25,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M25" s="10">
+      <c r="O25" s="10">
         <f>IF(A25="","",COUNTIF(Imagenes!A:A,A25))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="L26" s="10">
+      <c r="N26" s="10">
         <f>IF(A26="","",SUMIF(Variantes!A:A,A26,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M26" s="10">
+      <c r="O26" s="10">
         <f>IF(A26="","",COUNTIF(Imagenes!A:A,A26))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="L27" s="10">
+      <c r="N27" s="10">
         <f>IF(A27="","",SUMIF(Variantes!A:A,A27,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M27" s="10">
+      <c r="O27" s="10">
         <f>IF(A27="","",COUNTIF(Imagenes!A:A,A27))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="L28" s="10">
+      <c r="N28" s="10">
         <f>IF(A28="","",SUMIF(Variantes!A:A,A28,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M28" s="10">
+      <c r="O28" s="10">
         <f>IF(A28="","",COUNTIF(Imagenes!A:A,A28))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="L29" s="10">
+      <c r="N29" s="10">
         <f>IF(A29="","",SUMIF(Variantes!A:A,A29,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M29" s="10">
+      <c r="O29" s="10">
         <f>IF(A29="","",COUNTIF(Imagenes!A:A,A29))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="L30" s="10">
+      <c r="N30" s="10">
         <f>IF(A30="","",SUMIF(Variantes!A:A,A30,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M30" s="10">
+      <c r="O30" s="10">
         <f>IF(A30="","",COUNTIF(Imagenes!A:A,A30))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="L31" s="10">
+      <c r="N31" s="10">
         <f>IF(A31="","",SUMIF(Variantes!A:A,A31,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M31" s="10">
+      <c r="O31" s="10">
         <f>IF(A31="","",COUNTIF(Imagenes!A:A,A31))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="L32" s="10">
+      <c r="N32" s="10">
         <f>IF(A32="","",SUMIF(Variantes!A:A,A32,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M32" s="10">
+      <c r="O32" s="10">
         <f>IF(A32="","",COUNTIF(Imagenes!A:A,A32))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="L33" s="10">
+      <c r="N33" s="10">
         <f>IF(A33="","",SUMIF(Variantes!A:A,A33,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M33" s="10">
+      <c r="O33" s="10">
         <f>IF(A33="","",COUNTIF(Imagenes!A:A,A33))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="L34" s="10">
+      <c r="N34" s="10">
         <f>IF(A34="","",SUMIF(Variantes!A:A,A34,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M34" s="10">
+      <c r="O34" s="10">
         <f>IF(A34="","",COUNTIF(Imagenes!A:A,A34))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="L35" s="10">
+      <c r="N35" s="10">
         <f>IF(A35="","",SUMIF(Variantes!A:A,A35,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M35" s="10">
+      <c r="O35" s="10">
         <f>IF(A35="","",COUNTIF(Imagenes!A:A,A35))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="L36" s="10">
+      <c r="N36" s="10">
         <f>IF(A36="","",SUMIF(Variantes!A:A,A36,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M36" s="10">
+      <c r="O36" s="10">
         <f>IF(A36="","",COUNTIF(Imagenes!A:A,A36))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="L37" s="10">
+      <c r="N37" s="10">
         <f>IF(A37="","",SUMIF(Variantes!A:A,A37,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M37" s="10">
+      <c r="O37" s="10">
         <f>IF(A37="","",COUNTIF(Imagenes!A:A,A37))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="L38" s="10">
+      <c r="N38" s="10">
         <f>IF(A38="","",SUMIF(Variantes!A:A,A38,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M38" s="10">
+      <c r="O38" s="10">
         <f>IF(A38="","",COUNTIF(Imagenes!A:A,A38))</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="L39" s="10">
+      <c r="N39" s="10">
         <f>IF(A39="","",SUMIF(Variantes!A:A,A39,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M39" s="10">
+      <c r="O39" s="10">
         <f>IF(A39="","",COUNTIF(Imagenes!A:A,A39))</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="L40" s="10">
+      <c r="N40" s="10">
         <f>IF(A40="","",SUMIF(Variantes!A:A,A40,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M40" s="10">
+      <c r="O40" s="10">
         <f>IF(A40="","",COUNTIF(Imagenes!A:A,A40))</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="L41" s="10">
+      <c r="N41" s="10">
         <f>IF(A41="","",SUMIF(Variantes!A:A,A41,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M41" s="10">
+      <c r="O41" s="10">
         <f>IF(A41="","",COUNTIF(Imagenes!A:A,A41))</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="L42" s="10">
+      <c r="N42" s="10">
         <f>IF(A42="","",SUMIF(Variantes!A:A,A42,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M42" s="10">
+      <c r="O42" s="10">
         <f>IF(A42="","",COUNTIF(Imagenes!A:A,A42))</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="L43" s="10">
+      <c r="N43" s="10">
         <f>IF(A43="","",SUMIF(Variantes!A:A,A43,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M43" s="10">
+      <c r="O43" s="10">
         <f>IF(A43="","",COUNTIF(Imagenes!A:A,A43))</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="L44" s="10">
+      <c r="N44" s="10">
         <f>IF(A44="","",SUMIF(Variantes!A:A,A44,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M44" s="10">
+      <c r="O44" s="10">
         <f>IF(A44="","",COUNTIF(Imagenes!A:A,A44))</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="L45" s="10">
+      <c r="N45" s="10">
         <f>IF(A45="","",SUMIF(Variantes!A:A,A45,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M45" s="10">
+      <c r="O45" s="10">
         <f>IF(A45="","",COUNTIF(Imagenes!A:A,A45))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="L46" s="10">
+      <c r="N46" s="10">
         <f>IF(A46="","",SUMIF(Variantes!A:A,A46,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M46" s="10">
+      <c r="O46" s="10">
         <f>IF(A46="","",COUNTIF(Imagenes!A:A,A46))</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="L47" s="10">
+      <c r="N47" s="10">
         <f>IF(A47="","",SUMIF(Variantes!A:A,A47,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M47" s="10">
+      <c r="O47" s="10">
         <f>IF(A47="","",COUNTIF(Imagenes!A:A,A47))</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="L48" s="10">
+      <c r="N48" s="10">
         <f>IF(A48="","",SUMIF(Variantes!A:A,A48,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M48" s="10">
+      <c r="O48" s="10">
         <f>IF(A48="","",COUNTIF(Imagenes!A:A,A48))</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="L49" s="10">
+      <c r="N49" s="10">
         <f>IF(A49="","",SUMIF(Variantes!A:A,A49,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M49" s="10">
+      <c r="O49" s="10">
         <f>IF(A49="","",COUNTIF(Imagenes!A:A,A49))</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="L50" s="10">
+      <c r="N50" s="10">
         <f>IF(A50="","",SUMIF(Variantes!A:A,A50,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M50" s="10">
+      <c r="O50" s="10">
         <f>IF(A50="","",COUNTIF(Imagenes!A:A,A50))</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="L51" s="10">
+      <c r="N51" s="10">
         <f>IF(A51="","",SUMIF(Variantes!A:A,A51,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M51" s="10">
+      <c r="O51" s="10">
         <f>IF(A51="","",COUNTIF(Imagenes!A:A,A51))</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="L52" s="10">
+      <c r="N52" s="10">
         <f>IF(A52="","",SUMIF(Variantes!A:A,A52,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M52" s="10">
+      <c r="O52" s="10">
         <f>IF(A52="","",COUNTIF(Imagenes!A:A,A52))</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="L53" s="10">
+      <c r="N53" s="10">
         <f>IF(A53="","",SUMIF(Variantes!A:A,A53,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M53" s="10">
+      <c r="O53" s="10">
         <f>IF(A53="","",COUNTIF(Imagenes!A:A,A53))</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="L54" s="10">
+      <c r="N54" s="10">
         <f>IF(A54="","",SUMIF(Variantes!A:A,A54,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M54" s="10">
+      <c r="O54" s="10">
         <f>IF(A54="","",COUNTIF(Imagenes!A:A,A54))</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="L55" s="10">
+      <c r="N55" s="10">
         <f>IF(A55="","",SUMIF(Variantes!A:A,A55,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M55" s="10">
+      <c r="O55" s="10">
         <f>IF(A55="","",COUNTIF(Imagenes!A:A,A55))</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="L56" s="10">
+      <c r="N56" s="10">
         <f>IF(A56="","",SUMIF(Variantes!A:A,A56,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M56" s="10">
+      <c r="O56" s="10">
         <f>IF(A56="","",COUNTIF(Imagenes!A:A,A56))</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="L57" s="10">
+      <c r="N57" s="10">
         <f>IF(A57="","",SUMIF(Variantes!A:A,A57,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M57" s="10">
+      <c r="O57" s="10">
         <f>IF(A57="","",COUNTIF(Imagenes!A:A,A57))</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="L58" s="10">
+      <c r="N58" s="10">
         <f>IF(A58="","",SUMIF(Variantes!A:A,A58,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M58" s="10">
+      <c r="O58" s="10">
         <f>IF(A58="","",COUNTIF(Imagenes!A:A,A58))</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="L59" s="10">
+      <c r="N59" s="10">
         <f>IF(A59="","",SUMIF(Variantes!A:A,A59,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M59" s="10">
+      <c r="O59" s="10">
         <f>IF(A59="","",COUNTIF(Imagenes!A:A,A59))</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="L60" s="10">
+      <c r="N60" s="10">
         <f>IF(A60="","",SUMIF(Variantes!A:A,A60,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M60" s="10">
+      <c r="O60" s="10">
         <f>IF(A60="","",COUNTIF(Imagenes!A:A,A60))</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="L61" s="10">
+      <c r="N61" s="10">
         <f>IF(A61="","",SUMIF(Variantes!A:A,A61,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M61" s="10">
+      <c r="O61" s="10">
         <f>IF(A61="","",COUNTIF(Imagenes!A:A,A61))</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="L62" s="10">
+      <c r="N62" s="10">
         <f>IF(A62="","",SUMIF(Variantes!A:A,A62,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M62" s="10">
+      <c r="O62" s="10">
         <f>IF(A62="","",COUNTIF(Imagenes!A:A,A62))</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="L63" s="10">
+      <c r="N63" s="10">
         <f>IF(A63="","",SUMIF(Variantes!A:A,A63,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M63" s="10">
+      <c r="O63" s="10">
         <f>IF(A63="","",COUNTIF(Imagenes!A:A,A63))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="10">
+      <c r="N64" s="10">
         <f>IF(A64="","",SUMIF(Variantes!A:A,A64,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M64" s="10">
+      <c r="O64" s="10">
         <f>IF(A64="","",COUNTIF(Imagenes!A:A,A64))</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="10">
+      <c r="N65" s="10">
         <f>IF(A65="","",SUMIF(Variantes!A:A,A65,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M65" s="10">
+      <c r="O65" s="10">
         <f>IF(A65="","",COUNTIF(Imagenes!A:A,A65))</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="10">
+      <c r="N66" s="10">
         <f>IF(A66="","",SUMIF(Variantes!A:A,A66,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M66" s="10">
+      <c r="O66" s="10">
         <f>IF(A66="","",COUNTIF(Imagenes!A:A,A66))</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="10">
+      <c r="N67" s="10">
         <f>IF(A67="","",SUMIF(Variantes!A:A,A67,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M67" s="10">
+      <c r="O67" s="10">
         <f>IF(A67="","",COUNTIF(Imagenes!A:A,A67))</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="10">
+      <c r="N68" s="10">
         <f>IF(A68="","",SUMIF(Variantes!A:A,A68,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M68" s="10">
+      <c r="O68" s="10">
         <f>IF(A68="","",COUNTIF(Imagenes!A:A,A68))</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="10">
+      <c r="N69" s="10">
         <f>IF(A69="","",SUMIF(Variantes!A:A,A69,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M69" s="10">
+      <c r="O69" s="10">
         <f>IF(A69="","",COUNTIF(Imagenes!A:A,A69))</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="10">
+      <c r="N70" s="10">
         <f>IF(A70="","",SUMIF(Variantes!A:A,A70,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M70" s="10">
+      <c r="O70" s="10">
         <f>IF(A70="","",COUNTIF(Imagenes!A:A,A70))</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="L71" s="10">
+      <c r="N71" s="10">
         <f>IF(A71="","",SUMIF(Variantes!A:A,A71,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M71" s="10">
+      <c r="O71" s="10">
         <f>IF(A71="","",COUNTIF(Imagenes!A:A,A71))</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="10">
+      <c r="N72" s="10">
         <f>IF(A72="","",SUMIF(Variantes!A:A,A72,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M72" s="10">
+      <c r="O72" s="10">
         <f>IF(A72="","",COUNTIF(Imagenes!A:A,A72))</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="L73" s="10">
+      <c r="N73" s="10">
         <f>IF(A73="","",SUMIF(Variantes!A:A,A73,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M73" s="10">
+      <c r="O73" s="10">
         <f>IF(A73="","",COUNTIF(Imagenes!A:A,A73))</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="L74" s="10">
+      <c r="N74" s="10">
         <f>IF(A74="","",SUMIF(Variantes!A:A,A74,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M74" s="10">
+      <c r="O74" s="10">
         <f>IF(A74="","",COUNTIF(Imagenes!A:A,A74))</f>
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="L75" s="10">
+      <c r="N75" s="10">
         <f>IF(A75="","",SUMIF(Variantes!A:A,A75,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M75" s="10">
+      <c r="O75" s="10">
         <f>IF(A75="","",COUNTIF(Imagenes!A:A,A75))</f>
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="L76" s="10">
+      <c r="N76" s="10">
         <f>IF(A76="","",SUMIF(Variantes!A:A,A76,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M76" s="10">
+      <c r="O76" s="10">
         <f>IF(A76="","",COUNTIF(Imagenes!A:A,A76))</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="L77" s="10">
+      <c r="N77" s="10">
         <f>IF(A77="","",SUMIF(Variantes!A:A,A77,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M77" s="10">
+      <c r="O77" s="10">
         <f>IF(A77="","",COUNTIF(Imagenes!A:A,A77))</f>
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="L78" s="10">
+      <c r="N78" s="10">
         <f>IF(A78="","",SUMIF(Variantes!A:A,A78,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M78" s="10">
+      <c r="O78" s="10">
         <f>IF(A78="","",COUNTIF(Imagenes!A:A,A78))</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="L79" s="10">
+      <c r="N79" s="10">
         <f>IF(A79="","",SUMIF(Variantes!A:A,A79,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M79" s="10">
+      <c r="O79" s="10">
         <f>IF(A79="","",COUNTIF(Imagenes!A:A,A79))</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="L80" s="10">
+      <c r="N80" s="10">
         <f>IF(A80="","",SUMIF(Variantes!A:A,A80,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M80" s="10">
+      <c r="O80" s="10">
         <f>IF(A80="","",COUNTIF(Imagenes!A:A,A80))</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="L81" s="10">
+      <c r="N81" s="10">
         <f>IF(A81="","",SUMIF(Variantes!A:A,A81,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M81" s="10">
+      <c r="O81" s="10">
         <f>IF(A81="","",COUNTIF(Imagenes!A:A,A81))</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="L82" s="10">
+      <c r="N82" s="10">
         <f>IF(A82="","",SUMIF(Variantes!A:A,A82,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M82" s="10">
+      <c r="O82" s="10">
         <f>IF(A82="","",COUNTIF(Imagenes!A:A,A82))</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="L83" s="10">
+      <c r="N83" s="10">
         <f>IF(A83="","",SUMIF(Variantes!A:A,A83,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M83" s="10">
+      <c r="O83" s="10">
         <f>IF(A83="","",COUNTIF(Imagenes!A:A,A83))</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="L84" s="10">
+      <c r="N84" s="10">
         <f>IF(A84="","",SUMIF(Variantes!A:A,A84,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M84" s="10">
+      <c r="O84" s="10">
         <f>IF(A84="","",COUNTIF(Imagenes!A:A,A84))</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="L85" s="10">
+      <c r="N85" s="10">
         <f>IF(A85="","",SUMIF(Variantes!A:A,A85,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M85" s="10">
+      <c r="O85" s="10">
         <f>IF(A85="","",COUNTIF(Imagenes!A:A,A85))</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="L86" s="10">
+      <c r="N86" s="10">
         <f>IF(A86="","",SUMIF(Variantes!A:A,A86,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M86" s="10">
+      <c r="O86" s="10">
         <f>IF(A86="","",COUNTIF(Imagenes!A:A,A86))</f>
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="L87" s="10">
+      <c r="N87" s="10">
         <f>IF(A87="","",SUMIF(Variantes!A:A,A87,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M87" s="10">
+      <c r="O87" s="10">
         <f>IF(A87="","",COUNTIF(Imagenes!A:A,A87))</f>
         <v/>
       </c>
     </row>
     <row r="88">
-      <c r="L88" s="10">
+      <c r="N88" s="10">
         <f>IF(A88="","",SUMIF(Variantes!A:A,A88,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M88" s="10">
+      <c r="O88" s="10">
         <f>IF(A88="","",COUNTIF(Imagenes!A:A,A88))</f>
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="L89" s="10">
+      <c r="N89" s="10">
         <f>IF(A89="","",SUMIF(Variantes!A:A,A89,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M89" s="10">
+      <c r="O89" s="10">
         <f>IF(A89="","",COUNTIF(Imagenes!A:A,A89))</f>
         <v/>
       </c>
     </row>
     <row r="90">
-      <c r="L90" s="10">
+      <c r="N90" s="10">
         <f>IF(A90="","",SUMIF(Variantes!A:A,A90,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M90" s="10">
+      <c r="O90" s="10">
         <f>IF(A90="","",COUNTIF(Imagenes!A:A,A90))</f>
         <v/>
       </c>
     </row>
     <row r="91">
-      <c r="L91" s="10">
+      <c r="N91" s="10">
         <f>IF(A91="","",SUMIF(Variantes!A:A,A91,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M91" s="10">
+      <c r="O91" s="10">
         <f>IF(A91="","",COUNTIF(Imagenes!A:A,A91))</f>
         <v/>
       </c>
     </row>
     <row r="92">
-      <c r="L92" s="10">
+      <c r="N92" s="10">
         <f>IF(A92="","",SUMIF(Variantes!A:A,A92,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M92" s="10">
+      <c r="O92" s="10">
         <f>IF(A92="","",COUNTIF(Imagenes!A:A,A92))</f>
         <v/>
       </c>
     </row>
     <row r="93">
-      <c r="L93" s="10">
+      <c r="N93" s="10">
         <f>IF(A93="","",SUMIF(Variantes!A:A,A93,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M93" s="10">
+      <c r="O93" s="10">
         <f>IF(A93="","",COUNTIF(Imagenes!A:A,A93))</f>
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="L94" s="10">
+      <c r="N94" s="10">
         <f>IF(A94="","",SUMIF(Variantes!A:A,A94,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M94" s="10">
+      <c r="O94" s="10">
         <f>IF(A94="","",COUNTIF(Imagenes!A:A,A94))</f>
         <v/>
       </c>
     </row>
     <row r="95">
-      <c r="L95" s="10">
+      <c r="N95" s="10">
         <f>IF(A95="","",SUMIF(Variantes!A:A,A95,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M95" s="10">
+      <c r="O95" s="10">
         <f>IF(A95="","",COUNTIF(Imagenes!A:A,A95))</f>
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="L96" s="10">
+      <c r="N96" s="10">
         <f>IF(A96="","",SUMIF(Variantes!A:A,A96,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M96" s="10">
+      <c r="O96" s="10">
         <f>IF(A96="","",COUNTIF(Imagenes!A:A,A96))</f>
         <v/>
       </c>
     </row>
     <row r="97">
-      <c r="L97" s="10">
+      <c r="N97" s="10">
         <f>IF(A97="","",SUMIF(Variantes!A:A,A97,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M97" s="10">
+      <c r="O97" s="10">
         <f>IF(A97="","",COUNTIF(Imagenes!A:A,A97))</f>
         <v/>
       </c>
     </row>
     <row r="98">
-      <c r="L98" s="10">
+      <c r="N98" s="10">
         <f>IF(A98="","",SUMIF(Variantes!A:A,A98,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M98" s="10">
+      <c r="O98" s="10">
         <f>IF(A98="","",COUNTIF(Imagenes!A:A,A98))</f>
         <v/>
       </c>
     </row>
     <row r="99">
-      <c r="L99" s="10">
+      <c r="N99" s="10">
         <f>IF(A99="","",SUMIF(Variantes!A:A,A99,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M99" s="10">
+      <c r="O99" s="10">
         <f>IF(A99="","",COUNTIF(Imagenes!A:A,A99))</f>
         <v/>
       </c>
     </row>
     <row r="100">
-      <c r="L100" s="10">
+      <c r="N100" s="10">
         <f>IF(A100="","",SUMIF(Variantes!A:A,A100,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M100" s="10">
+      <c r="O100" s="10">
         <f>IF(A100="","",COUNTIF(Imagenes!A:A,A100))</f>
         <v/>
       </c>
     </row>
     <row r="101">
-      <c r="L101" s="10">
+      <c r="N101" s="10">
         <f>IF(A101="","",SUMIF(Variantes!A:A,A101,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M101" s="10">
+      <c r="O101" s="10">
         <f>IF(A101="","",COUNTIF(Imagenes!A:A,A101))</f>
         <v/>
       </c>
     </row>
     <row r="102">
-      <c r="L102" s="10">
+      <c r="N102" s="10">
         <f>IF(A102="","",SUMIF(Variantes!A:A,A102,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M102" s="10">
+      <c r="O102" s="10">
         <f>IF(A102="","",COUNTIF(Imagenes!A:A,A102))</f>
         <v/>
       </c>
     </row>
     <row r="103">
-      <c r="L103" s="10">
+      <c r="N103" s="10">
         <f>IF(A103="","",SUMIF(Variantes!A:A,A103,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M103" s="10">
+      <c r="O103" s="10">
         <f>IF(A103="","",COUNTIF(Imagenes!A:A,A103))</f>
         <v/>
       </c>
     </row>
     <row r="104">
-      <c r="L104" s="10">
+      <c r="N104" s="10">
         <f>IF(A104="","",SUMIF(Variantes!A:A,A104,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M104" s="10">
+      <c r="O104" s="10">
         <f>IF(A104="","",COUNTIF(Imagenes!A:A,A104))</f>
         <v/>
       </c>
     </row>
     <row r="105">
-      <c r="L105" s="10">
+      <c r="N105" s="10">
         <f>IF(A105="","",SUMIF(Variantes!A:A,A105,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M105" s="10">
+      <c r="O105" s="10">
         <f>IF(A105="","",COUNTIF(Imagenes!A:A,A105))</f>
         <v/>
       </c>
     </row>
     <row r="106">
-      <c r="L106" s="10">
+      <c r="N106" s="10">
         <f>IF(A106="","",SUMIF(Variantes!A:A,A106,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M106" s="10">
+      <c r="O106" s="10">
         <f>IF(A106="","",COUNTIF(Imagenes!A:A,A106))</f>
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="L107" s="10">
+      <c r="N107" s="10">
         <f>IF(A107="","",SUMIF(Variantes!A:A,A107,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M107" s="10">
+      <c r="O107" s="10">
         <f>IF(A107="","",COUNTIF(Imagenes!A:A,A107))</f>
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="L108" s="10">
+      <c r="N108" s="10">
         <f>IF(A108="","",SUMIF(Variantes!A:A,A108,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M108" s="10">
+      <c r="O108" s="10">
         <f>IF(A108="","",COUNTIF(Imagenes!A:A,A108))</f>
         <v/>
       </c>
     </row>
     <row r="109">
-      <c r="L109" s="10">
+      <c r="N109" s="10">
         <f>IF(A109="","",SUMIF(Variantes!A:A,A109,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M109" s="10">
+      <c r="O109" s="10">
         <f>IF(A109="","",COUNTIF(Imagenes!A:A,A109))</f>
         <v/>
       </c>
     </row>
     <row r="110">
-      <c r="L110" s="10">
+      <c r="N110" s="10">
         <f>IF(A110="","",SUMIF(Variantes!A:A,A110,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M110" s="10">
+      <c r="O110" s="10">
         <f>IF(A110="","",COUNTIF(Imagenes!A:A,A110))</f>
         <v/>
       </c>
     </row>
     <row r="111">
-      <c r="L111" s="10">
+      <c r="N111" s="10">
         <f>IF(A111="","",SUMIF(Variantes!A:A,A111,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M111" s="10">
+      <c r="O111" s="10">
         <f>IF(A111="","",COUNTIF(Imagenes!A:A,A111))</f>
         <v/>
       </c>
     </row>
     <row r="112">
-      <c r="L112" s="10">
+      <c r="N112" s="10">
         <f>IF(A112="","",SUMIF(Variantes!A:A,A112,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M112" s="10">
+      <c r="O112" s="10">
         <f>IF(A112="","",COUNTIF(Imagenes!A:A,A112))</f>
         <v/>
       </c>
     </row>
     <row r="113">
-      <c r="L113" s="10">
+      <c r="N113" s="10">
         <f>IF(A113="","",SUMIF(Variantes!A:A,A113,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M113" s="10">
+      <c r="O113" s="10">
         <f>IF(A113="","",COUNTIF(Imagenes!A:A,A113))</f>
         <v/>
       </c>
     </row>
     <row r="114">
-      <c r="L114" s="10">
+      <c r="N114" s="10">
         <f>IF(A114="","",SUMIF(Variantes!A:A,A114,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M114" s="10">
+      <c r="O114" s="10">
         <f>IF(A114="","",COUNTIF(Imagenes!A:A,A114))</f>
         <v/>
       </c>
     </row>
     <row r="115">
-      <c r="L115" s="10">
+      <c r="N115" s="10">
         <f>IF(A115="","",SUMIF(Variantes!A:A,A115,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M115" s="10">
+      <c r="O115" s="10">
         <f>IF(A115="","",COUNTIF(Imagenes!A:A,A115))</f>
         <v/>
       </c>
     </row>
     <row r="116">
-      <c r="L116" s="10">
+      <c r="N116" s="10">
         <f>IF(A116="","",SUMIF(Variantes!A:A,A116,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M116" s="10">
+      <c r="O116" s="10">
         <f>IF(A116="","",COUNTIF(Imagenes!A:A,A116))</f>
         <v/>
       </c>
     </row>
     <row r="117">
-      <c r="L117" s="10">
+      <c r="N117" s="10">
         <f>IF(A117="","",SUMIF(Variantes!A:A,A117,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M117" s="10">
+      <c r="O117" s="10">
         <f>IF(A117="","",COUNTIF(Imagenes!A:A,A117))</f>
         <v/>
       </c>
     </row>
     <row r="118">
-      <c r="L118" s="10">
+      <c r="N118" s="10">
         <f>IF(A118="","",SUMIF(Variantes!A:A,A118,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M118" s="10">
+      <c r="O118" s="10">
         <f>IF(A118="","",COUNTIF(Imagenes!A:A,A118))</f>
         <v/>
       </c>
     </row>
     <row r="119">
-      <c r="L119" s="10">
+      <c r="N119" s="10">
         <f>IF(A119="","",SUMIF(Variantes!A:A,A119,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M119" s="10">
+      <c r="O119" s="10">
         <f>IF(A119="","",COUNTIF(Imagenes!A:A,A119))</f>
         <v/>
       </c>
     </row>
     <row r="120">
-      <c r="L120" s="10">
+      <c r="N120" s="10">
         <f>IF(A120="","",SUMIF(Variantes!A:A,A120,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M120" s="10">
+      <c r="O120" s="10">
         <f>IF(A120="","",COUNTIF(Imagenes!A:A,A120))</f>
         <v/>
       </c>
     </row>
     <row r="121">
-      <c r="L121" s="10">
+      <c r="N121" s="10">
         <f>IF(A121="","",SUMIF(Variantes!A:A,A121,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M121" s="10">
+      <c r="O121" s="10">
         <f>IF(A121="","",COUNTIF(Imagenes!A:A,A121))</f>
         <v/>
       </c>
     </row>
     <row r="122">
-      <c r="L122" s="10">
+      <c r="N122" s="10">
         <f>IF(A122="","",SUMIF(Variantes!A:A,A122,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M122" s="10">
+      <c r="O122" s="10">
         <f>IF(A122="","",COUNTIF(Imagenes!A:A,A122))</f>
         <v/>
       </c>
     </row>
     <row r="123">
-      <c r="L123" s="10">
+      <c r="N123" s="10">
         <f>IF(A123="","",SUMIF(Variantes!A:A,A123,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M123" s="10">
+      <c r="O123" s="10">
         <f>IF(A123="","",COUNTIF(Imagenes!A:A,A123))</f>
         <v/>
       </c>
     </row>
     <row r="124">
-      <c r="L124" s="10">
+      <c r="N124" s="10">
         <f>IF(A124="","",SUMIF(Variantes!A:A,A124,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M124" s="10">
+      <c r="O124" s="10">
         <f>IF(A124="","",COUNTIF(Imagenes!A:A,A124))</f>
         <v/>
       </c>
     </row>
     <row r="125">
-      <c r="L125" s="10">
+      <c r="N125" s="10">
         <f>IF(A125="","",SUMIF(Variantes!A:A,A125,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M125" s="10">
+      <c r="O125" s="10">
         <f>IF(A125="","",COUNTIF(Imagenes!A:A,A125))</f>
         <v/>
       </c>
     </row>
     <row r="126">
-      <c r="L126" s="10">
+      <c r="N126" s="10">
         <f>IF(A126="","",SUMIF(Variantes!A:A,A126,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M126" s="10">
+      <c r="O126" s="10">
         <f>IF(A126="","",COUNTIF(Imagenes!A:A,A126))</f>
         <v/>
       </c>
     </row>
     <row r="127">
-      <c r="L127" s="10">
+      <c r="N127" s="10">
         <f>IF(A127="","",SUMIF(Variantes!A:A,A127,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M127" s="10">
+      <c r="O127" s="10">
         <f>IF(A127="","",COUNTIF(Imagenes!A:A,A127))</f>
         <v/>
       </c>
     </row>
     <row r="128">
-      <c r="L128" s="10">
+      <c r="N128" s="10">
         <f>IF(A128="","",SUMIF(Variantes!A:A,A128,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M128" s="10">
+      <c r="O128" s="10">
         <f>IF(A128="","",COUNTIF(Imagenes!A:A,A128))</f>
         <v/>
       </c>
     </row>
     <row r="129">
-      <c r="L129" s="10">
+      <c r="N129" s="10">
         <f>IF(A129="","",SUMIF(Variantes!A:A,A129,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M129" s="10">
+      <c r="O129" s="10">
         <f>IF(A129="","",COUNTIF(Imagenes!A:A,A129))</f>
         <v/>
       </c>
     </row>
     <row r="130">
-      <c r="L130" s="10">
+      <c r="N130" s="10">
         <f>IF(A130="","",SUMIF(Variantes!A:A,A130,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M130" s="10">
+      <c r="O130" s="10">
         <f>IF(A130="","",COUNTIF(Imagenes!A:A,A130))</f>
         <v/>
       </c>
     </row>
     <row r="131">
-      <c r="L131" s="10">
+      <c r="N131" s="10">
         <f>IF(A131="","",SUMIF(Variantes!A:A,A131,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M131" s="10">
+      <c r="O131" s="10">
         <f>IF(A131="","",COUNTIF(Imagenes!A:A,A131))</f>
         <v/>
       </c>
     </row>
     <row r="132">
-      <c r="L132" s="10">
+      <c r="N132" s="10">
         <f>IF(A132="","",SUMIF(Variantes!A:A,A132,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M132" s="10">
+      <c r="O132" s="10">
         <f>IF(A132="","",COUNTIF(Imagenes!A:A,A132))</f>
         <v/>
       </c>
     </row>
     <row r="133">
-      <c r="L133" s="10">
+      <c r="N133" s="10">
         <f>IF(A133="","",SUMIF(Variantes!A:A,A133,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M133" s="10">
+      <c r="O133" s="10">
         <f>IF(A133="","",COUNTIF(Imagenes!A:A,A133))</f>
         <v/>
       </c>
     </row>
     <row r="134">
-      <c r="L134" s="10">
+      <c r="N134" s="10">
         <f>IF(A134="","",SUMIF(Variantes!A:A,A134,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M134" s="10">
+      <c r="O134" s="10">
         <f>IF(A134="","",COUNTIF(Imagenes!A:A,A134))</f>
         <v/>
       </c>
     </row>
     <row r="135">
-      <c r="L135" s="10">
+      <c r="N135" s="10">
         <f>IF(A135="","",SUMIF(Variantes!A:A,A135,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M135" s="10">
+      <c r="O135" s="10">
         <f>IF(A135="","",COUNTIF(Imagenes!A:A,A135))</f>
         <v/>
       </c>
     </row>
     <row r="136">
-      <c r="L136" s="10">
+      <c r="N136" s="10">
         <f>IF(A136="","",SUMIF(Variantes!A:A,A136,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M136" s="10">
+      <c r="O136" s="10">
         <f>IF(A136="","",COUNTIF(Imagenes!A:A,A136))</f>
         <v/>
       </c>
     </row>
     <row r="137">
-      <c r="L137" s="10">
+      <c r="N137" s="10">
         <f>IF(A137="","",SUMIF(Variantes!A:A,A137,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M137" s="10">
+      <c r="O137" s="10">
         <f>IF(A137="","",COUNTIF(Imagenes!A:A,A137))</f>
         <v/>
       </c>
     </row>
     <row r="138">
-      <c r="L138" s="10">
+      <c r="N138" s="10">
         <f>IF(A138="","",SUMIF(Variantes!A:A,A138,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M138" s="10">
+      <c r="O138" s="10">
         <f>IF(A138="","",COUNTIF(Imagenes!A:A,A138))</f>
         <v/>
       </c>
     </row>
     <row r="139">
-      <c r="L139" s="10">
+      <c r="N139" s="10">
         <f>IF(A139="","",SUMIF(Variantes!A:A,A139,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M139" s="10">
+      <c r="O139" s="10">
         <f>IF(A139="","",COUNTIF(Imagenes!A:A,A139))</f>
         <v/>
       </c>
     </row>
     <row r="140">
-      <c r="L140" s="10">
+      <c r="N140" s="10">
         <f>IF(A140="","",SUMIF(Variantes!A:A,A140,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M140" s="10">
+      <c r="O140" s="10">
         <f>IF(A140="","",COUNTIF(Imagenes!A:A,A140))</f>
         <v/>
       </c>
     </row>
     <row r="141">
-      <c r="L141" s="10">
+      <c r="N141" s="10">
         <f>IF(A141="","",SUMIF(Variantes!A:A,A141,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M141" s="10">
+      <c r="O141" s="10">
         <f>IF(A141="","",COUNTIF(Imagenes!A:A,A141))</f>
         <v/>
       </c>
     </row>
     <row r="142">
-      <c r="L142" s="10">
+      <c r="N142" s="10">
         <f>IF(A142="","",SUMIF(Variantes!A:A,A142,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M142" s="10">
+      <c r="O142" s="10">
         <f>IF(A142="","",COUNTIF(Imagenes!A:A,A142))</f>
         <v/>
       </c>
     </row>
     <row r="143">
-      <c r="L143" s="10">
+      <c r="N143" s="10">
         <f>IF(A143="","",SUMIF(Variantes!A:A,A143,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M143" s="10">
+      <c r="O143" s="10">
         <f>IF(A143="","",COUNTIF(Imagenes!A:A,A143))</f>
         <v/>
       </c>
     </row>
     <row r="144">
-      <c r="L144" s="10">
+      <c r="N144" s="10">
         <f>IF(A144="","",SUMIF(Variantes!A:A,A144,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M144" s="10">
+      <c r="O144" s="10">
         <f>IF(A144="","",COUNTIF(Imagenes!A:A,A144))</f>
         <v/>
       </c>
     </row>
     <row r="145">
-      <c r="L145" s="10">
+      <c r="N145" s="10">
         <f>IF(A145="","",SUMIF(Variantes!A:A,A145,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M145" s="10">
+      <c r="O145" s="10">
         <f>IF(A145="","",COUNTIF(Imagenes!A:A,A145))</f>
         <v/>
       </c>
     </row>
     <row r="146">
-      <c r="L146" s="10">
+      <c r="N146" s="10">
         <f>IF(A146="","",SUMIF(Variantes!A:A,A146,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M146" s="10">
+      <c r="O146" s="10">
         <f>IF(A146="","",COUNTIF(Imagenes!A:A,A146))</f>
         <v/>
       </c>
     </row>
     <row r="147">
-      <c r="L147" s="10">
+      <c r="N147" s="10">
         <f>IF(A147="","",SUMIF(Variantes!A:A,A147,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M147" s="10">
+      <c r="O147" s="10">
         <f>IF(A147="","",COUNTIF(Imagenes!A:A,A147))</f>
         <v/>
       </c>
     </row>
     <row r="148">
-      <c r="L148" s="10">
+      <c r="N148" s="10">
         <f>IF(A148="","",SUMIF(Variantes!A:A,A148,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M148" s="10">
+      <c r="O148" s="10">
         <f>IF(A148="","",COUNTIF(Imagenes!A:A,A148))</f>
         <v/>
       </c>
     </row>
     <row r="149">
-      <c r="L149" s="10">
+      <c r="N149" s="10">
         <f>IF(A149="","",SUMIF(Variantes!A:A,A149,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M149" s="10">
+      <c r="O149" s="10">
         <f>IF(A149="","",COUNTIF(Imagenes!A:A,A149))</f>
         <v/>
       </c>
     </row>
     <row r="150">
-      <c r="L150" s="10">
+      <c r="N150" s="10">
         <f>IF(A150="","",SUMIF(Variantes!A:A,A150,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M150" s="10">
+      <c r="O150" s="10">
         <f>IF(A150="","",COUNTIF(Imagenes!A:A,A150))</f>
         <v/>
       </c>
     </row>
     <row r="151">
-      <c r="L151" s="10">
+      <c r="N151" s="10">
         <f>IF(A151="","",SUMIF(Variantes!A:A,A151,Variantes!D:D))</f>
         <v/>
       </c>
-      <c r="M151" s="10">
+      <c r="O151" s="10">
         <f>IF(A151="","",COUNTIF(Imagenes!A:A,A151))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
-      <formula1>=Listas!$A$2:$A$100</formula1>
+      <formula1>=Listas!$A$2:$A$20</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
-      <formula1>"SI,NO"</formula1>
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>=Listas!$C$2:$C$60</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>=Marcas!$A$2:$A$50</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>"SI,NO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2481,7 +2570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2515,47 +2604,22 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>e2</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>c1-NEG</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Negro</t>
+          <t>e2</t>
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>c1</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>c1-CAF</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
-      <formula1>=Productos!$A$2:$A$1000</formula1>
+      <formula1>=Productos!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2603,7 +2667,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>e2</t>
         </is>
       </c>
       <c r="B2" s="7" t="n">
@@ -2611,19 +2675,19 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/.../c1-1.jpg</t>
+          <t>https://res.cloudinary.com/.../e2-1.jpg</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>c1-1.jpg</t>
+          <t>e2-1.jpg</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
-      <formula1>=Productos!$A$2:$A$1000</formula1>
+      <formula1>=Productos!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2637,7 +2701,87 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>logo_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Cartago</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>San Fermín</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Mesacé</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Al Torno</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Sybec</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Natural V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Cheval</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2669,18 +2813,11 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Pesos por dólar para mostrar precios en USD. Valor de ejemplo: actualícenlo con la tasa que usan para cotizar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>La celda amarilla es el valor que ustedes editan.</t>
+          <t>Pesos por dólar para mostrar precios en USD. Se actualiza cada 8 días.</t>
         </is>
       </c>
     </row>
@@ -2689,16 +2826,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="3" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2707,6 +2847,17 @@
           <t>categorias</t>
         </is>
       </c>
+      <c r="B1" s="6" t="inlineStr"/>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>subcategorias</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>de la categoría</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
@@ -2714,46 +2865,250 @@
           <t>Monturas</t>
         </is>
       </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Sillas</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Monturas</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Riendas y cabezadas</t>
+          <t>Equino</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Tereques</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Monturas</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Aperos y arneses</t>
+          <t>Jinete</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Galápagos</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Monturas</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Correas</t>
+          <t>Cuidado del caballo</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Monturas</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Bolsos</t>
+          <t>Caninos</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Cabeza</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Equino</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Billeteras</t>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Alfombras</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Equino</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Mascotas</t>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Alforjas</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Equino</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Correaje</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Equino</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Tarabas</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Equino</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Sombreros</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Jinete</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Marroquinería</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Jinete</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Bisutería</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Jinete</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Aseo</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Cuidado del caballo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Suplementos</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Cuidado del caballo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Accesorios</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Cuidado del caballo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Pecheras</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Caninos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Collares</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Caninos</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Traíllas</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Caninos</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Bozales</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Caninos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar panel de administración con usuarios y contraseña
- /admin (carga aparte): productos, colores y stock, fotos a Cloudinary,
  tasa del dólar, marcas, usuarios y historial de cambios
- Apps Script: sesiones validadas en el servidor, contraseñas con hash y sal
  en propiedades privadas, bloqueo por intentos, candado de escritura,
  firma de Cloudinary y menú para armar la hoja y crear usuarios
- Modo de prueba local sin Sheet (solo en desarrollo)
- Se retira la plantilla Excel: la hoja la arma el propio script

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cartago_Inventario_Plantilla.xlsx
+++ b/docs/Cartago_Inventario_Plantilla.xlsx
@@ -212,176 +212,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>JCS Emprende</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Código corto y único: letra + número (m1, e1, j1). No se repite ni se cambia.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Elige de la lista (pestaña Listas).</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Elige de la lista. Debe corresponder a la categoría (ver pestaña Listas).</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Elige de la lista (pestaña Marcas). Cada producto muestra el logo de su marca.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Pesos colombianos, sin puntos ni signo. 0 o vacío = Precio a consultar.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>Opcional. Precio fijo en dólares. Vacío = se convierte con la tasa de Configuracion.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>SI = se ve en la página. NO = escondido.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>SI = aparece en Productos destacados de la página de inicio.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>SI = el cliente puede escribir el bordado o el detalle que quiere.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>Texto de ayuda que ve el cliente en el campo de personalización.</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>Opcional. Texto resaltado en la ficha del producto.</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>Se calcula solo: suma del stock de todos los colores en Variantes.</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>Se calcula solo: cuántas fotos tiene el producto en Imagenes.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>JCS Emprende</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>El id del producto, tal como está en Productos.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Código único de esta variante: id + 3 letras del color (j2-NEG). Sin colores: el mismo id.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Nombre del color. Vacío si el producto no maneja colores.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Unidades disponibles de este color. 0 = agotado.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>JCS Emprende</author>
-  </authors>
-  <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>1 = foto de portada; luego 2, 3...</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Link de la foto en Cloudinary (lo escribe JCS Emprende).</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Nombre del archivo en la carpeta de Drive, para ubicarlo (e2-1.jpg).</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>JCS Emprende</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Nombre de la marca tal como se escribe en Productos.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Opcional. Link del logo. Cartago, San Fermín y Mesacé ya vienen incluidos en la página.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>JCS Emprende</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Categorías que se pueden elegir en Productos.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Subcategorías que se pueden elegir en Productos.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2560,7 +2390,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2623,7 +2452,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2691,7 +2519,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2771,7 +2598,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3114,6 +2940,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>